<commit_message>
Update 'events.xlsx' to add the inauguration in 2025.
</commit_message>
<xml_diff>
--- a/data/aux/events.xlsx
+++ b/data/aux/events.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="73">
   <si>
     <t xml:space="preserve">Changepoint</t>
   </si>
@@ -212,6 +212,12 @@
   </si>
   <si>
     <t xml:space="preserve">2025-01-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inauguration and first days of the second Trump administration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-01-20</t>
   </si>
   <si>
     <t xml:space="preserve">2025-09-22 00:00:01</t>
@@ -243,7 +249,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -265,14 +271,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -317,13 +315,9 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -351,8 +345,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="65.62"/>
   </cols>
@@ -384,366 +378,392 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="E5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="E9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="E10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="E12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="E13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="3" t="s">
+      <c r="A14" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="G14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="H14" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="E15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D15" s="3" t="s">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="C16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="H15" s="2" t="s">
+      <c r="F16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>